<commit_message>
Resolved the Health Insurance page
</commit_message>
<xml_diff>
--- a/HealthInsurance.xlsx
+++ b/HealthInsurance.xlsx
@@ -12,9 +12,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
-    <t/>
+    <t>Health insurance</t>
+  </si>
+  <si>
+    <t>Health insurance Plans for Family</t>
+  </si>
+  <si>
+    <t>Health Insurance Premium Calculator</t>
+  </si>
+  <si>
+    <t>Health Insurance for Parents</t>
+  </si>
+  <si>
+    <t>Senior Citizen Health Insurance</t>
+  </si>
+  <si>
+    <t>Section 80D</t>
+  </si>
+  <si>
+    <t>Arogya Sanjeevani Health Insurance</t>
   </si>
 </sst>
 </file>
@@ -59,7 +77,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -69,52 +87,32 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>